<commit_message>
Update off day, OT, and shift plans CSV and Excel files; modify employee search view for improved functionality
</commit_message>
<xml_diff>
--- a/public/assets/excel/off_day_plans.xlsx
+++ b/public/assets/excel/off_day_plans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo LOQ\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3197676-6EDD-4B57-97C2-60414EB944FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B92C7CA7-4752-4319-AC2B-FD40999AEB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="off_day_plans" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="21">
   <si>
     <t>Name</t>
   </si>
@@ -77,6 +77,12 @@
   </si>
   <si>
     <t>VD</t>
+  </si>
+  <si>
+    <t>9.15 AM</t>
+  </si>
+  <si>
+    <t>6.30 PM</t>
   </si>
 </sst>
 </file>
@@ -114,7 +120,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,29 +424,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.81640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -456,18 +462,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1">
-        <v>0.375</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0.75</v>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="E2">
         <v>15</v>
@@ -482,18 +488,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="1">
-        <v>0.375</v>
-      </c>
-      <c r="D3" s="1">
-        <v>0.75</v>
+      <c r="C3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="E3">
         <v>15</v>
@@ -508,18 +514,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="1">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="D4" s="1">
-        <v>0.70833333333333337</v>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="E4">
         <v>12</v>
@@ -534,18 +540,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="1">
-        <v>0.29166666666666669</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0.75</v>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="E5">
         <v>15</v>
@@ -560,18 +566,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>17</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1">
-        <v>0.25</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0.79166666666666696</v>
+      <c r="C6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="E6">
         <v>20</v>

</xml_diff>